<commit_message>
Gerichte Excel erweitert um Scores und Nachtisse
</commit_message>
<xml_diff>
--- a/data/CaterNow_Data_master.xlsx
+++ b/data/CaterNow_Data_master.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/benedicthorbelt/Documents/Github/uni-caternow-booking-service/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA38C41F-D53E-C948-BD99-FBE34979B334}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AE3C7AF-FB2A-734C-A38D-24B4260D9B5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="160" yWindow="940" windowWidth="30020" windowHeight="19100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="160" yWindow="940" windowWidth="25180" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MainData" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <sheet name="Desserts" sheetId="4" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">MainData!$B$1:$P$128</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">MainData!$B$1:$P$137</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1370" uniqueCount="497">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1418" uniqueCount="511">
   <si>
     <t>productTitle</t>
   </si>
@@ -1532,6 +1532,48 @@
   <si>
     <t>img_link</t>
   </si>
+  <si>
+    <t>Baklava</t>
+  </si>
+  <si>
+    <t>Knuspriges Blätterteiggebäck mit gehackten Pistazien und Walnüssen, großzügig getränkt in Rosenwasser-Honigsirup</t>
+  </si>
+  <si>
+    <t>Kunafa</t>
+  </si>
+  <si>
+    <t>Warmes Engelshaar-Gebäck gefüllt mit cremigem Frischkäse, übergossen mit Zuckersirup und garniert mit gemahlenen Pistazien</t>
+  </si>
+  <si>
+    <t>Muhallebi</t>
+  </si>
+  <si>
+    <t>Zarter Milchreis-Pudding parfümiert mit Rosenwasser und Orangenblüten, garniert mit gemahlenen Pistazien und getrockneten Rosenblättern</t>
+  </si>
+  <si>
+    <t>Halva mit Pistazien</t>
+  </si>
+  <si>
+    <t>Traditionelle Sesampaste-Konfekt mit gerösteten Pistazien und einem Hauch Kardamom, serviert mit frischen Feigen</t>
+  </si>
+  <si>
+    <t>Mango Sticky Rice</t>
+  </si>
+  <si>
+    <t>Klebreis mit frischer Alphonso-Mango und cremiger Kokosmilchsauce, verfeinert mit geröstetem Sesam</t>
+  </si>
+  <si>
+    <t>Matcha Panna Cotta</t>
+  </si>
+  <si>
+    <t>Seidige Panna Cotta mit hochwertigem japanischen Matcha, serviert mit einem Yuzu-Gelee und weißer Schokolade</t>
+  </si>
+  <si>
+    <t>Black Sesame Mochi</t>
+  </si>
+  <si>
+    <t>Zarte Reiskuchen gefüllt mit cremiger schwarzer Sesampaste und Azuki-Bohnencreme, leicht gepudert mit Stärke</t>
+  </si>
 </sst>
 </file>
 
@@ -2821,7 +2863,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:X930"/>
@@ -2953,7 +2995,7 @@
       <c r="W2" s="5"/>
       <c r="X2" s="5"/>
     </row>
-    <row r="3" spans="1:24" ht="13.75" customHeight="1">
+    <row r="3" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A3" s="31">
         <v>102</v>
       </c>
@@ -3001,7 +3043,7 @@
       <c r="W3" s="5"/>
       <c r="X3" s="5"/>
     </row>
-    <row r="4" spans="1:24" ht="13.75" customHeight="1">
+    <row r="4" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A4" s="31">
         <v>103</v>
       </c>
@@ -3055,7 +3097,7 @@
       <c r="W4" s="5"/>
       <c r="X4" s="5"/>
     </row>
-    <row r="5" spans="1:24" ht="13.75" customHeight="1">
+    <row r="5" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A5" s="31">
         <v>104</v>
       </c>
@@ -3109,7 +3151,7 @@
       <c r="W5" s="5"/>
       <c r="X5" s="5"/>
     </row>
-    <row r="6" spans="1:24" ht="13.75" customHeight="1">
+    <row r="6" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A6" s="31">
         <v>105</v>
       </c>
@@ -3163,7 +3205,7 @@
       <c r="W6" s="5"/>
       <c r="X6" s="5"/>
     </row>
-    <row r="7" spans="1:24" ht="13.75" customHeight="1">
+    <row r="7" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A7" s="31">
         <v>106</v>
       </c>
@@ -3217,7 +3259,7 @@
       <c r="W7" s="5"/>
       <c r="X7" s="5"/>
     </row>
-    <row r="8" spans="1:24" ht="13.75" customHeight="1">
+    <row r="8" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A8" s="31">
         <v>107</v>
       </c>
@@ -3271,7 +3313,7 @@
       <c r="W8" s="5"/>
       <c r="X8" s="5"/>
     </row>
-    <row r="9" spans="1:24" ht="13.75" customHeight="1">
+    <row r="9" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A9" s="31">
         <v>108</v>
       </c>
@@ -3323,7 +3365,7 @@
       <c r="W9" s="5"/>
       <c r="X9" s="5"/>
     </row>
-    <row r="10" spans="1:24" ht="13.75" customHeight="1">
+    <row r="10" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A10" s="31">
         <v>109</v>
       </c>
@@ -3377,7 +3419,7 @@
       <c r="W10" s="5"/>
       <c r="X10" s="5"/>
     </row>
-    <row r="11" spans="1:24" ht="13.75" customHeight="1">
+    <row r="11" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A11" s="31">
         <v>110</v>
       </c>
@@ -3427,7 +3469,7 @@
       <c r="W11" s="5"/>
       <c r="X11" s="5"/>
     </row>
-    <row r="12" spans="1:24" ht="13.75" customHeight="1">
+    <row r="12" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A12" s="31">
         <v>111</v>
       </c>
@@ -3477,7 +3519,7 @@
       <c r="W12" s="5"/>
       <c r="X12" s="5"/>
     </row>
-    <row r="13" spans="1:24" ht="13.75" customHeight="1">
+    <row r="13" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A13" s="31">
         <v>112</v>
       </c>
@@ -3527,7 +3569,7 @@
       <c r="W13" s="5"/>
       <c r="X13" s="5"/>
     </row>
-    <row r="14" spans="1:24" ht="13.75" customHeight="1">
+    <row r="14" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A14" s="31">
         <v>113</v>
       </c>
@@ -3579,7 +3621,7 @@
       <c r="W14" s="5"/>
       <c r="X14" s="5"/>
     </row>
-    <row r="15" spans="1:24" ht="13.75" customHeight="1">
+    <row r="15" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A15" s="31">
         <v>114</v>
       </c>
@@ -3629,7 +3671,7 @@
       <c r="W15" s="5"/>
       <c r="X15" s="5"/>
     </row>
-    <row r="16" spans="1:24" ht="13.75" customHeight="1">
+    <row r="16" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A16" s="31">
         <v>115</v>
       </c>
@@ -3679,7 +3721,7 @@
       <c r="W16" s="5"/>
       <c r="X16" s="5"/>
     </row>
-    <row r="17" spans="1:24" ht="13.75" customHeight="1">
+    <row r="17" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A17" s="31">
         <v>116</v>
       </c>
@@ -3731,7 +3773,7 @@
       <c r="W17" s="5"/>
       <c r="X17" s="5"/>
     </row>
-    <row r="18" spans="1:24" ht="13.75" customHeight="1">
+    <row r="18" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A18" s="31">
         <v>117</v>
       </c>
@@ -3785,7 +3827,7 @@
       <c r="W18" s="5"/>
       <c r="X18" s="5"/>
     </row>
-    <row r="19" spans="1:24" ht="13.75" customHeight="1">
+    <row r="19" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A19" s="31">
         <v>118</v>
       </c>
@@ -3839,7 +3881,7 @@
       <c r="W19" s="5"/>
       <c r="X19" s="5"/>
     </row>
-    <row r="20" spans="1:24" ht="13.75" customHeight="1">
+    <row r="20" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A20" s="31">
         <v>119</v>
       </c>
@@ -3891,7 +3933,7 @@
       <c r="W20" s="5"/>
       <c r="X20" s="5"/>
     </row>
-    <row r="21" spans="1:24" ht="13.75" customHeight="1">
+    <row r="21" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A21" s="31">
         <v>120</v>
       </c>
@@ -3945,7 +3987,7 @@
       <c r="W21" s="5"/>
       <c r="X21" s="5"/>
     </row>
-    <row r="22" spans="1:24" ht="13.75" customHeight="1">
+    <row r="22" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A22" s="31">
         <v>121</v>
       </c>
@@ -3999,7 +4041,7 @@
       <c r="W22" s="5"/>
       <c r="X22" s="5"/>
     </row>
-    <row r="23" spans="1:24" ht="13.75" customHeight="1">
+    <row r="23" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A23" s="31">
         <v>122</v>
       </c>
@@ -4051,7 +4093,7 @@
       <c r="W23" s="5"/>
       <c r="X23" s="5"/>
     </row>
-    <row r="24" spans="1:24" ht="13.75" customHeight="1">
+    <row r="24" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A24" s="31">
         <v>123</v>
       </c>
@@ -4105,7 +4147,7 @@
       <c r="W24" s="5"/>
       <c r="X24" s="5"/>
     </row>
-    <row r="25" spans="1:24" ht="13.75" customHeight="1">
+    <row r="25" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A25" s="31">
         <v>124</v>
       </c>
@@ -4159,7 +4201,7 @@
       <c r="W25" s="5"/>
       <c r="X25" s="5"/>
     </row>
-    <row r="26" spans="1:24" ht="13.75" customHeight="1">
+    <row r="26" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A26" s="31">
         <v>125</v>
       </c>
@@ -4213,7 +4255,7 @@
       <c r="W26" s="5"/>
       <c r="X26" s="5"/>
     </row>
-    <row r="27" spans="1:24" ht="13.75" customHeight="1">
+    <row r="27" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A27" s="31">
         <v>126</v>
       </c>
@@ -4267,7 +4309,7 @@
       <c r="W27" s="5"/>
       <c r="X27" s="5"/>
     </row>
-    <row r="28" spans="1:24" ht="13.75" customHeight="1">
+    <row r="28" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A28" s="31">
         <v>127</v>
       </c>
@@ -4321,7 +4363,7 @@
       <c r="W28" s="5"/>
       <c r="X28" s="5"/>
     </row>
-    <row r="29" spans="1:24" ht="13.75" customHeight="1">
+    <row r="29" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A29" s="31">
         <v>128</v>
       </c>
@@ -4375,7 +4417,7 @@
       <c r="W29" s="5"/>
       <c r="X29" s="5"/>
     </row>
-    <row r="30" spans="1:24" ht="13.75" customHeight="1">
+    <row r="30" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A30" s="31">
         <v>129</v>
       </c>
@@ -4610,7 +4652,9 @@
       <c r="H34" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="I34" s="5"/>
+      <c r="I34" s="21" t="s">
+        <v>278</v>
+      </c>
       <c r="J34" s="24">
         <v>0.5</v>
       </c>
@@ -4662,7 +4706,9 @@
       <c r="H35" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="I35" s="5"/>
+      <c r="I35" s="21" t="s">
+        <v>278</v>
+      </c>
       <c r="J35" s="24">
         <v>0.5</v>
       </c>
@@ -4793,7 +4839,7 @@
       <c r="W37" s="5"/>
       <c r="X37" s="5"/>
     </row>
-    <row r="38" spans="1:24" ht="13.75" customHeight="1">
+    <row r="38" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A38" s="31">
         <v>137</v>
       </c>
@@ -4845,7 +4891,7 @@
       <c r="W38" s="5"/>
       <c r="X38" s="5"/>
     </row>
-    <row r="39" spans="1:24" ht="13.75" customHeight="1">
+    <row r="39" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A39" s="31">
         <v>138</v>
       </c>
@@ -4897,7 +4943,7 @@
       <c r="W39" s="5"/>
       <c r="X39" s="5"/>
     </row>
-    <row r="40" spans="1:24" ht="13.75" customHeight="1">
+    <row r="40" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A40" s="31">
         <v>139</v>
       </c>
@@ -4951,7 +4997,7 @@
       <c r="W40" s="5"/>
       <c r="X40" s="5"/>
     </row>
-    <row r="41" spans="1:24" ht="13.75" customHeight="1">
+    <row r="41" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A41" s="31">
         <v>140</v>
       </c>
@@ -5003,7 +5049,7 @@
       <c r="W41" s="5"/>
       <c r="X41" s="5"/>
     </row>
-    <row r="42" spans="1:24" ht="13.75" customHeight="1">
+    <row r="42" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A42" s="31">
         <v>141</v>
       </c>
@@ -5053,7 +5099,7 @@
       <c r="W42" s="5"/>
       <c r="X42" s="5"/>
     </row>
-    <row r="43" spans="1:24" ht="13.75" customHeight="1">
+    <row r="43" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A43" s="31">
         <v>142</v>
       </c>
@@ -5105,7 +5151,7 @@
       <c r="W43" s="5"/>
       <c r="X43" s="5"/>
     </row>
-    <row r="44" spans="1:24" ht="13.75" customHeight="1">
+    <row r="44" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A44" s="31">
         <v>143</v>
       </c>
@@ -5155,7 +5201,7 @@
       <c r="W44" s="5"/>
       <c r="X44" s="5"/>
     </row>
-    <row r="45" spans="1:24" ht="13.75" customHeight="1">
+    <row r="45" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A45" s="31">
         <v>144</v>
       </c>
@@ -5363,7 +5409,7 @@
       <c r="W48" s="5"/>
       <c r="X48" s="5"/>
     </row>
-    <row r="49" spans="1:24" ht="13.75" customHeight="1">
+    <row r="49" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A49" s="31">
         <v>148</v>
       </c>
@@ -5415,7 +5461,7 @@
       <c r="W49" s="5"/>
       <c r="X49" s="5"/>
     </row>
-    <row r="50" spans="1:24" ht="13.75" customHeight="1">
+    <row r="50" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A50" s="31">
         <v>149</v>
       </c>
@@ -5467,7 +5513,7 @@
       <c r="W50" s="5"/>
       <c r="X50" s="5"/>
     </row>
-    <row r="51" spans="1:24" ht="13.75" customHeight="1">
+    <row r="51" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A51" s="31">
         <v>150</v>
       </c>
@@ -5519,7 +5565,7 @@
       <c r="W51" s="5"/>
       <c r="X51" s="5"/>
     </row>
-    <row r="52" spans="1:24" ht="13.75" customHeight="1">
+    <row r="52" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A52" s="31">
         <v>151</v>
       </c>
@@ -5571,7 +5617,7 @@
       <c r="W52" s="5"/>
       <c r="X52" s="5"/>
     </row>
-    <row r="53" spans="1:24" ht="15.75" customHeight="1">
+    <row r="53" spans="1:24" ht="15.75" hidden="1" customHeight="1">
       <c r="A53" s="31">
         <v>152</v>
       </c>
@@ -5613,7 +5659,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:24" ht="15.75" customHeight="1">
+    <row r="54" spans="1:24" ht="15.75" hidden="1" customHeight="1">
       <c r="A54" s="31">
         <v>153</v>
       </c>
@@ -5655,7 +5701,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:24" ht="15.75" customHeight="1">
+    <row r="55" spans="1:24" ht="15.75" hidden="1" customHeight="1">
       <c r="A55" s="31">
         <v>154</v>
       </c>
@@ -5695,7 +5741,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:24" ht="15.75" customHeight="1">
+    <row r="56" spans="1:24" ht="15.75" hidden="1" customHeight="1">
       <c r="A56" s="31">
         <v>155</v>
       </c>
@@ -5737,7 +5783,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:24" ht="15.75" customHeight="1">
+    <row r="57" spans="1:24" ht="15.75" hidden="1" customHeight="1">
       <c r="A57" s="31">
         <v>156</v>
       </c>
@@ -5779,7 +5825,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:24" ht="15.75" customHeight="1">
+    <row r="58" spans="1:24" ht="15.75" hidden="1" customHeight="1">
       <c r="A58" s="31">
         <v>157</v>
       </c>
@@ -5821,7 +5867,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:24" ht="15.75" customHeight="1">
+    <row r="59" spans="1:24" ht="15.75" hidden="1" customHeight="1">
       <c r="A59" s="31">
         <v>158</v>
       </c>
@@ -5949,7 +5995,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:24" ht="15.75" customHeight="1">
+    <row r="62" spans="1:24" ht="15.75" hidden="1" customHeight="1">
       <c r="A62" s="31">
         <v>161</v>
       </c>
@@ -5991,7 +6037,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="63" spans="1:24" ht="15.75" customHeight="1">
+    <row r="63" spans="1:24" ht="15.75" hidden="1" customHeight="1">
       <c r="A63" s="31">
         <v>162</v>
       </c>
@@ -6031,7 +6077,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="64" spans="1:24" ht="15.75" customHeight="1">
+    <row r="64" spans="1:24" ht="15.75" hidden="1" customHeight="1">
       <c r="A64" s="31">
         <v>163</v>
       </c>
@@ -6073,7 +6119,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:24" ht="13.75" customHeight="1">
+    <row r="65" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A65" s="31">
         <v>164</v>
       </c>
@@ -6125,7 +6171,7 @@
       <c r="W65" s="5"/>
       <c r="X65" s="5"/>
     </row>
-    <row r="66" spans="1:24" ht="13.75" customHeight="1">
+    <row r="66" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A66" s="31">
         <v>165</v>
       </c>
@@ -6177,7 +6223,7 @@
       <c r="W66" s="5"/>
       <c r="X66" s="5"/>
     </row>
-    <row r="67" spans="1:24" ht="13.75" customHeight="1">
+    <row r="67" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A67" s="31">
         <v>166</v>
       </c>
@@ -6229,7 +6275,7 @@
       <c r="W67" s="5"/>
       <c r="X67" s="5"/>
     </row>
-    <row r="68" spans="1:24" ht="13.75" customHeight="1">
+    <row r="68" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A68" s="31">
         <v>167</v>
       </c>
@@ -6281,7 +6327,7 @@
       <c r="W68" s="5"/>
       <c r="X68" s="5"/>
     </row>
-    <row r="69" spans="1:24" ht="13.75" customHeight="1">
+    <row r="69" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A69" s="31">
         <v>168</v>
       </c>
@@ -6333,7 +6379,7 @@
       <c r="W69" s="5"/>
       <c r="X69" s="5"/>
     </row>
-    <row r="70" spans="1:24" ht="13.75" customHeight="1">
+    <row r="70" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A70" s="31">
         <v>169</v>
       </c>
@@ -6385,7 +6431,7 @@
       <c r="W70" s="5"/>
       <c r="X70" s="5"/>
     </row>
-    <row r="71" spans="1:24" ht="13.75" customHeight="1">
+    <row r="71" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A71" s="31">
         <v>170</v>
       </c>
@@ -6437,7 +6483,7 @@
       <c r="W71" s="5"/>
       <c r="X71" s="5"/>
     </row>
-    <row r="72" spans="1:24" ht="13.75" customHeight="1">
+    <row r="72" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A72" s="31">
         <v>171</v>
       </c>
@@ -6489,7 +6535,7 @@
       <c r="W72" s="5"/>
       <c r="X72" s="5"/>
     </row>
-    <row r="73" spans="1:24" ht="13.75" customHeight="1">
+    <row r="73" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A73" s="31">
         <v>172</v>
       </c>
@@ -6541,7 +6587,7 @@
       <c r="W73" s="5"/>
       <c r="X73" s="5"/>
     </row>
-    <row r="74" spans="1:24" ht="13.75" customHeight="1">
+    <row r="74" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A74" s="31">
         <v>173</v>
       </c>
@@ -6593,7 +6639,7 @@
       <c r="W74" s="5"/>
       <c r="X74" s="5"/>
     </row>
-    <row r="75" spans="1:24" ht="13.75" customHeight="1">
+    <row r="75" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A75" s="31">
         <v>174</v>
       </c>
@@ -6645,7 +6691,7 @@
       <c r="W75" s="5"/>
       <c r="X75" s="5"/>
     </row>
-    <row r="76" spans="1:24" ht="13.75" customHeight="1">
+    <row r="76" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A76" s="31">
         <v>175</v>
       </c>
@@ -6697,7 +6743,7 @@
       <c r="W76" s="5"/>
       <c r="X76" s="5"/>
     </row>
-    <row r="77" spans="1:24" ht="13.75" customHeight="1">
+    <row r="77" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A77" s="31">
         <v>176</v>
       </c>
@@ -6749,7 +6795,7 @@
       <c r="W77" s="5"/>
       <c r="X77" s="5"/>
     </row>
-    <row r="78" spans="1:24" ht="13.75" customHeight="1">
+    <row r="78" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A78" s="31">
         <v>177</v>
       </c>
@@ -6801,7 +6847,7 @@
       <c r="W78" s="5"/>
       <c r="X78" s="5"/>
     </row>
-    <row r="79" spans="1:24" ht="13.75" customHeight="1">
+    <row r="79" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A79" s="31">
         <v>178</v>
       </c>
@@ -6853,7 +6899,7 @@
       <c r="W79" s="5"/>
       <c r="X79" s="5"/>
     </row>
-    <row r="80" spans="1:24" ht="13.75" customHeight="1">
+    <row r="80" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A80" s="31">
         <v>179</v>
       </c>
@@ -6907,7 +6953,7 @@
       <c r="W80" s="5"/>
       <c r="X80" s="5"/>
     </row>
-    <row r="81" spans="1:24" ht="13.75" customHeight="1">
+    <row r="81" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A81" s="31">
         <v>180</v>
       </c>
@@ -6961,7 +7007,7 @@
       <c r="W81" s="5"/>
       <c r="X81" s="5"/>
     </row>
-    <row r="82" spans="1:24" ht="13.75" customHeight="1">
+    <row r="82" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A82" s="31">
         <v>181</v>
       </c>
@@ -7013,7 +7059,7 @@
       <c r="W82" s="5"/>
       <c r="X82" s="5"/>
     </row>
-    <row r="83" spans="1:24" ht="13.75" customHeight="1">
+    <row r="83" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A83" s="31">
         <v>182</v>
       </c>
@@ -7065,7 +7111,7 @@
       <c r="W83" s="5"/>
       <c r="X83" s="5"/>
     </row>
-    <row r="84" spans="1:24" ht="13.75" customHeight="1">
+    <row r="84" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A84" s="31">
         <v>183</v>
       </c>
@@ -7117,7 +7163,7 @@
       <c r="W84" s="5"/>
       <c r="X84" s="5"/>
     </row>
-    <row r="85" spans="1:24" ht="13.75" customHeight="1">
+    <row r="85" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A85" s="31">
         <v>184</v>
       </c>
@@ -7169,7 +7215,7 @@
       <c r="W85" s="5"/>
       <c r="X85" s="5"/>
     </row>
-    <row r="86" spans="1:24" ht="13.75" customHeight="1">
+    <row r="86" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A86" s="31">
         <v>185</v>
       </c>
@@ -7219,7 +7265,7 @@
       <c r="W86" s="5"/>
       <c r="X86" s="5"/>
     </row>
-    <row r="87" spans="1:24" ht="13.75" customHeight="1">
+    <row r="87" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A87" s="31">
         <v>186</v>
       </c>
@@ -7269,7 +7315,7 @@
       <c r="W87" s="5"/>
       <c r="X87" s="5"/>
     </row>
-    <row r="88" spans="1:24" ht="13.75" customHeight="1">
+    <row r="88" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A88" s="31">
         <v>187</v>
       </c>
@@ -7321,7 +7367,7 @@
       <c r="W88" s="5"/>
       <c r="X88" s="5"/>
     </row>
-    <row r="89" spans="1:24" ht="13.75" customHeight="1">
+    <row r="89" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A89" s="31">
         <v>188</v>
       </c>
@@ -7373,7 +7419,7 @@
       <c r="W89" s="5"/>
       <c r="X89" s="5"/>
     </row>
-    <row r="90" spans="1:24" ht="13.75" customHeight="1">
+    <row r="90" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A90" s="31">
         <v>189</v>
       </c>
@@ -7425,7 +7471,7 @@
       <c r="W90" s="5"/>
       <c r="X90" s="5"/>
     </row>
-    <row r="91" spans="1:24" ht="13.75" customHeight="1">
+    <row r="91" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A91" s="31">
         <v>190</v>
       </c>
@@ -7477,7 +7523,7 @@
       <c r="W91" s="5"/>
       <c r="X91" s="5"/>
     </row>
-    <row r="92" spans="1:24" ht="13.75" customHeight="1">
+    <row r="92" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A92" s="31">
         <v>191</v>
       </c>
@@ -7529,7 +7575,7 @@
       <c r="W92" s="5"/>
       <c r="X92" s="5"/>
     </row>
-    <row r="93" spans="1:24" ht="13.75" customHeight="1">
+    <row r="93" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A93" s="31">
         <v>192</v>
       </c>
@@ -7581,7 +7627,7 @@
       <c r="W93" s="5"/>
       <c r="X93" s="5"/>
     </row>
-    <row r="94" spans="1:24" ht="13.75" customHeight="1">
+    <row r="94" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A94" s="31">
         <v>193</v>
       </c>
@@ -7633,7 +7679,7 @@
       <c r="W94" s="5"/>
       <c r="X94" s="5"/>
     </row>
-    <row r="95" spans="1:24" ht="13.75" customHeight="1">
+    <row r="95" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A95" s="31">
         <v>194</v>
       </c>
@@ -7683,7 +7729,7 @@
       <c r="W95" s="5"/>
       <c r="X95" s="5"/>
     </row>
-    <row r="96" spans="1:24" ht="13.75" customHeight="1">
+    <row r="96" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A96" s="31">
         <v>195</v>
       </c>
@@ -7735,7 +7781,7 @@
       <c r="W96" s="5"/>
       <c r="X96" s="5"/>
     </row>
-    <row r="97" spans="1:24" ht="13.75" customHeight="1">
+    <row r="97" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A97" s="31">
         <v>196</v>
       </c>
@@ -7787,7 +7833,7 @@
       <c r="W97" s="5"/>
       <c r="X97" s="5"/>
     </row>
-    <row r="98" spans="1:24" ht="13.75" customHeight="1">
+    <row r="98" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A98" s="31">
         <v>197</v>
       </c>
@@ -7839,7 +7885,7 @@
       <c r="W98" s="5"/>
       <c r="X98" s="5"/>
     </row>
-    <row r="99" spans="1:24" ht="13.75" customHeight="1">
+    <row r="99" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A99" s="31">
         <v>198</v>
       </c>
@@ -7891,7 +7937,7 @@
       <c r="W99" s="5"/>
       <c r="X99" s="5"/>
     </row>
-    <row r="100" spans="1:24" ht="13.75" customHeight="1">
+    <row r="100" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A100" s="31">
         <v>199</v>
       </c>
@@ -7943,7 +7989,7 @@
       <c r="W100" s="5"/>
       <c r="X100" s="5"/>
     </row>
-    <row r="101" spans="1:24" ht="13.75" customHeight="1">
+    <row r="101" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A101" s="31">
         <v>200</v>
       </c>
@@ -7995,7 +8041,7 @@
       <c r="W101" s="5"/>
       <c r="X101" s="5"/>
     </row>
-    <row r="102" spans="1:24" ht="13.75" customHeight="1">
+    <row r="102" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A102" s="31">
         <v>201</v>
       </c>
@@ -8047,7 +8093,7 @@
       <c r="W102" s="5"/>
       <c r="X102" s="5"/>
     </row>
-    <row r="103" spans="1:24" ht="13.75" customHeight="1">
+    <row r="103" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A103" s="31">
         <v>202</v>
       </c>
@@ -8099,7 +8145,7 @@
       <c r="W103" s="5"/>
       <c r="X103" s="5"/>
     </row>
-    <row r="104" spans="1:24" ht="13.75" customHeight="1">
+    <row r="104" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A104" s="31">
         <v>203</v>
       </c>
@@ -8151,7 +8197,7 @@
       <c r="W104" s="5"/>
       <c r="X104" s="5"/>
     </row>
-    <row r="105" spans="1:24" ht="13.75" customHeight="1">
+    <row r="105" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A105" s="31">
         <v>204</v>
       </c>
@@ -8201,7 +8247,7 @@
       <c r="W105" s="5"/>
       <c r="X105" s="5"/>
     </row>
-    <row r="106" spans="1:24" ht="13.75" customHeight="1">
+    <row r="106" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A106" s="31">
         <v>205</v>
       </c>
@@ -8251,7 +8297,7 @@
       <c r="W106" s="5"/>
       <c r="X106" s="5"/>
     </row>
-    <row r="107" spans="1:24" ht="13.75" customHeight="1">
+    <row r="107" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A107" s="31">
         <v>206</v>
       </c>
@@ -8303,7 +8349,7 @@
       <c r="W107" s="5"/>
       <c r="X107" s="5"/>
     </row>
-    <row r="108" spans="1:24" ht="13.75" customHeight="1">
+    <row r="108" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A108" s="31">
         <v>207</v>
       </c>
@@ -8355,7 +8401,7 @@
       <c r="W108" s="5"/>
       <c r="X108" s="5"/>
     </row>
-    <row r="109" spans="1:24" ht="13.75" customHeight="1">
+    <row r="109" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A109" s="31">
         <v>208</v>
       </c>
@@ -8407,7 +8453,7 @@
       <c r="W109" s="5"/>
       <c r="X109" s="5"/>
     </row>
-    <row r="110" spans="1:24" ht="13.75" customHeight="1">
+    <row r="110" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A110" s="31">
         <v>209</v>
       </c>
@@ -8459,7 +8505,7 @@
       <c r="W110" s="5"/>
       <c r="X110" s="5"/>
     </row>
-    <row r="111" spans="1:24" ht="13.75" customHeight="1">
+    <row r="111" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A111" s="31">
         <v>210</v>
       </c>
@@ -8511,7 +8557,7 @@
       <c r="W111" s="5"/>
       <c r="X111" s="5"/>
     </row>
-    <row r="112" spans="1:24" ht="13.75" customHeight="1">
+    <row r="112" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A112" s="31">
         <v>211</v>
       </c>
@@ -8563,7 +8609,7 @@
       <c r="W112" s="5"/>
       <c r="X112" s="5"/>
     </row>
-    <row r="113" spans="1:24" ht="13.75" customHeight="1">
+    <row r="113" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A113" s="31">
         <v>212</v>
       </c>
@@ -8615,7 +8661,7 @@
       <c r="W113" s="5"/>
       <c r="X113" s="5"/>
     </row>
-    <row r="114" spans="1:24" ht="13.75" customHeight="1">
+    <row r="114" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A114" s="31">
         <v>213</v>
       </c>
@@ -8667,7 +8713,7 @@
       <c r="W114" s="5"/>
       <c r="X114" s="5"/>
     </row>
-    <row r="115" spans="1:24" ht="13.75" customHeight="1">
+    <row r="115" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A115" s="31">
         <v>214</v>
       </c>
@@ -8719,7 +8765,7 @@
       <c r="W115" s="5"/>
       <c r="X115" s="5"/>
     </row>
-    <row r="116" spans="1:24" ht="13.75" customHeight="1">
+    <row r="116" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A116" s="31">
         <v>215</v>
       </c>
@@ -8771,7 +8817,7 @@
       <c r="W116" s="5"/>
       <c r="X116" s="5"/>
     </row>
-    <row r="117" spans="1:24" ht="13.75" customHeight="1">
+    <row r="117" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A117" s="31">
         <v>216</v>
       </c>
@@ -8823,7 +8869,7 @@
       <c r="W117" s="5"/>
       <c r="X117" s="5"/>
     </row>
-    <row r="118" spans="1:24" ht="13.75" customHeight="1">
+    <row r="118" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A118" s="31">
         <v>217</v>
       </c>
@@ -8875,7 +8921,7 @@
       <c r="W118" s="5"/>
       <c r="X118" s="5"/>
     </row>
-    <row r="119" spans="1:24" ht="13.75" customHeight="1">
+    <row r="119" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A119" s="31">
         <v>218</v>
       </c>
@@ -8925,7 +8971,7 @@
       <c r="W119" s="5"/>
       <c r="X119" s="5"/>
     </row>
-    <row r="120" spans="1:24" ht="13.75" customHeight="1">
+    <row r="120" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A120" s="31">
         <v>219</v>
       </c>
@@ -8975,7 +9021,7 @@
       <c r="W120" s="5"/>
       <c r="X120" s="5"/>
     </row>
-    <row r="121" spans="1:24" ht="13.75" customHeight="1">
+    <row r="121" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A121" s="31">
         <v>220</v>
       </c>
@@ -9025,7 +9071,7 @@
       <c r="W121" s="5"/>
       <c r="X121" s="5"/>
     </row>
-    <row r="122" spans="1:24" ht="13.75" customHeight="1">
+    <row r="122" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A122" s="31">
         <v>221</v>
       </c>
@@ -9075,7 +9121,7 @@
       <c r="W122" s="5"/>
       <c r="X122" s="5"/>
     </row>
-    <row r="123" spans="1:24" ht="13.75" customHeight="1">
+    <row r="123" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A123" s="31">
         <v>222</v>
       </c>
@@ -9127,7 +9173,7 @@
       <c r="W123" s="5"/>
       <c r="X123" s="5"/>
     </row>
-    <row r="124" spans="1:24" ht="13.75" customHeight="1">
+    <row r="124" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A124" s="31">
         <v>223</v>
       </c>
@@ -9179,7 +9225,7 @@
       <c r="W124" s="5"/>
       <c r="X124" s="5"/>
     </row>
-    <row r="125" spans="1:24" ht="13.75" customHeight="1">
+    <row r="125" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A125" s="31">
         <v>224</v>
       </c>
@@ -9231,7 +9277,7 @@
       <c r="W125" s="5"/>
       <c r="X125" s="5"/>
     </row>
-    <row r="126" spans="1:24" ht="13.75" customHeight="1">
+    <row r="126" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A126" s="31">
         <v>225</v>
       </c>
@@ -9281,7 +9327,7 @@
       <c r="W126" s="5"/>
       <c r="X126" s="5"/>
     </row>
-    <row r="127" spans="1:24" ht="13.75" customHeight="1">
+    <row r="127" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A127" s="31">
         <v>226</v>
       </c>
@@ -9331,7 +9377,7 @@
       <c r="W127" s="5"/>
       <c r="X127" s="5"/>
     </row>
-    <row r="128" spans="1:24" ht="13.75" customHeight="1">
+    <row r="128" spans="1:24" ht="13.75" hidden="1" customHeight="1">
       <c r="A128" s="31">
         <v>227</v>
       </c>
@@ -9385,19 +9431,45 @@
     </row>
     <row r="129" spans="1:24" ht="13.75" customHeight="1">
       <c r="A129" s="9"/>
-      <c r="B129" s="8"/>
-      <c r="C129" s="8"/>
-      <c r="D129" s="8"/>
-      <c r="E129" s="8"/>
-      <c r="F129" s="8"/>
-      <c r="G129" s="8"/>
-      <c r="H129" s="8"/>
-      <c r="I129" s="8"/>
-      <c r="J129" s="5"/>
-      <c r="K129" s="5"/>
-      <c r="L129" s="5"/>
-      <c r="M129" s="5"/>
-      <c r="N129" s="5"/>
+      <c r="B129" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="C129" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="D129" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="E129" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="F129" s="9">
+        <v>3.9</v>
+      </c>
+      <c r="G129" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H129" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="I129" s="21" t="s">
+        <v>279</v>
+      </c>
+      <c r="J129" s="5">
+        <v>0.7</v>
+      </c>
+      <c r="K129" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="L129" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="M129" s="5">
+        <v>0.9</v>
+      </c>
+      <c r="N129" s="5">
+        <v>0</v>
+      </c>
       <c r="O129" s="5"/>
       <c r="P129" s="5"/>
       <c r="Q129" s="5"/>
@@ -9411,19 +9483,45 @@
     </row>
     <row r="130" spans="1:24" ht="13.75" customHeight="1">
       <c r="A130" s="9"/>
-      <c r="B130" s="8"/>
-      <c r="C130" s="8"/>
-      <c r="D130" s="8"/>
-      <c r="E130" s="8"/>
-      <c r="F130" s="8"/>
-      <c r="G130" s="8"/>
-      <c r="H130" s="8"/>
-      <c r="I130" s="8"/>
-      <c r="J130" s="5"/>
-      <c r="K130" s="5"/>
-      <c r="L130" s="5"/>
-      <c r="M130" s="5"/>
-      <c r="N130" s="5"/>
+      <c r="B130" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="C130" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="D130" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="E130" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="F130" s="9">
+        <v>3.9</v>
+      </c>
+      <c r="G130" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H130" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="I130" s="8" t="s">
+        <v>279</v>
+      </c>
+      <c r="J130" s="5">
+        <v>0.6</v>
+      </c>
+      <c r="K130" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="L130" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="M130" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="N130" s="5">
+        <v>0</v>
+      </c>
       <c r="O130" s="5"/>
       <c r="P130" s="5"/>
       <c r="Q130" s="5"/>
@@ -9437,19 +9535,43 @@
     </row>
     <row r="131" spans="1:24" ht="13.75" customHeight="1">
       <c r="A131" s="9"/>
-      <c r="B131" s="8"/>
-      <c r="C131" s="8"/>
-      <c r="D131" s="8"/>
-      <c r="E131" s="8"/>
-      <c r="F131" s="8"/>
-      <c r="G131" s="8"/>
-      <c r="H131" s="8"/>
-      <c r="I131" s="8"/>
-      <c r="J131" s="5"/>
-      <c r="K131" s="5"/>
-      <c r="L131" s="5"/>
-      <c r="M131" s="5"/>
-      <c r="N131" s="5"/>
+      <c r="B131" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="C131" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="D131" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="E131" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="F131" s="9">
+        <v>2.9</v>
+      </c>
+      <c r="G131" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H131" s="12"/>
+      <c r="I131" s="21" t="s">
+        <v>275</v>
+      </c>
+      <c r="J131" s="5">
+        <v>0.6</v>
+      </c>
+      <c r="K131" s="5">
+        <v>0.4</v>
+      </c>
+      <c r="L131" s="5">
+        <v>0.3</v>
+      </c>
+      <c r="M131" s="5">
+        <v>0.9</v>
+      </c>
+      <c r="N131" s="5">
+        <v>0</v>
+      </c>
       <c r="O131" s="5"/>
       <c r="P131" s="5"/>
       <c r="Q131" s="5"/>
@@ -9463,19 +9585,45 @@
     </row>
     <row r="132" spans="1:24" ht="13.75" customHeight="1">
       <c r="A132" s="9"/>
-      <c r="B132" s="8"/>
-      <c r="C132" s="8"/>
-      <c r="D132" s="8"/>
-      <c r="E132" s="8"/>
-      <c r="F132" s="8"/>
-      <c r="G132" s="8"/>
-      <c r="H132" s="8"/>
-      <c r="I132" s="8"/>
-      <c r="J132" s="5"/>
-      <c r="K132" s="5"/>
-      <c r="L132" s="5"/>
-      <c r="M132" s="5"/>
-      <c r="N132" s="5"/>
+      <c r="B132" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="C132" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="D132" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="E132" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="F132" s="9">
+        <v>3.9</v>
+      </c>
+      <c r="G132" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="H132" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="I132" s="21" t="s">
+        <v>279</v>
+      </c>
+      <c r="J132" s="5">
+        <v>0.6</v>
+      </c>
+      <c r="K132" s="5">
+        <v>0.3</v>
+      </c>
+      <c r="L132" s="5">
+        <v>0.3</v>
+      </c>
+      <c r="M132" s="5">
+        <v>0.4</v>
+      </c>
+      <c r="N132" s="5">
+        <v>0</v>
+      </c>
       <c r="O132" s="5"/>
       <c r="P132" s="5"/>
       <c r="Q132" s="5"/>
@@ -9489,19 +9637,43 @@
     </row>
     <row r="133" spans="1:24" ht="13.75" customHeight="1">
       <c r="A133" s="9"/>
-      <c r="B133" s="8"/>
-      <c r="C133" s="8"/>
-      <c r="D133" s="8"/>
-      <c r="E133" s="8"/>
-      <c r="F133" s="8"/>
-      <c r="G133" s="8"/>
-      <c r="H133" s="8"/>
-      <c r="I133" s="8"/>
-      <c r="J133" s="5"/>
-      <c r="K133" s="5"/>
-      <c r="L133" s="5"/>
-      <c r="M133" s="5"/>
-      <c r="N133" s="5"/>
+      <c r="B133" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="C133" s="8" t="s">
+        <v>268</v>
+      </c>
+      <c r="D133" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="E133" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="F133" s="9">
+        <v>3.9</v>
+      </c>
+      <c r="G133" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="H133" s="12"/>
+      <c r="I133" s="21" t="s">
+        <v>275</v>
+      </c>
+      <c r="J133" s="5">
+        <v>0.4</v>
+      </c>
+      <c r="K133" s="5">
+        <v>0.2</v>
+      </c>
+      <c r="L133" s="5">
+        <v>0.2</v>
+      </c>
+      <c r="M133" s="5">
+        <v>0.8</v>
+      </c>
+      <c r="N133" s="5">
+        <v>0</v>
+      </c>
       <c r="O133" s="5"/>
       <c r="P133" s="5"/>
       <c r="Q133" s="5"/>
@@ -9515,19 +9687,45 @@
     </row>
     <row r="134" spans="1:24" ht="13.75" customHeight="1">
       <c r="A134" s="9"/>
-      <c r="B134" s="8"/>
-      <c r="C134" s="8"/>
-      <c r="D134" s="8"/>
-      <c r="E134" s="8"/>
-      <c r="F134" s="8"/>
-      <c r="G134" s="8"/>
-      <c r="H134" s="8"/>
-      <c r="I134" s="8"/>
-      <c r="J134" s="5"/>
-      <c r="K134" s="5"/>
-      <c r="L134" s="5"/>
-      <c r="M134" s="5"/>
-      <c r="N134" s="5"/>
+      <c r="B134" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="C134" s="8" t="s">
+        <v>244</v>
+      </c>
+      <c r="D134" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="E134" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="F134" s="9">
+        <v>3.9</v>
+      </c>
+      <c r="G134" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H134" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="I134" s="21" t="s">
+        <v>278</v>
+      </c>
+      <c r="J134" s="5">
+        <v>0.8</v>
+      </c>
+      <c r="K134" s="5">
+        <v>0.4</v>
+      </c>
+      <c r="L134" s="5">
+        <v>0.4</v>
+      </c>
+      <c r="M134" s="5">
+        <v>0.2</v>
+      </c>
+      <c r="N134" s="5">
+        <v>0</v>
+      </c>
       <c r="O134" s="5"/>
       <c r="P134" s="5"/>
       <c r="Q134" s="5"/>
@@ -9541,19 +9739,45 @@
     </row>
     <row r="135" spans="1:24" ht="13.75" customHeight="1">
       <c r="A135" s="9"/>
-      <c r="B135" s="8"/>
-      <c r="C135" s="8"/>
-      <c r="D135" s="8"/>
-      <c r="E135" s="8"/>
-      <c r="F135" s="8"/>
-      <c r="G135" s="8"/>
-      <c r="H135" s="8"/>
-      <c r="I135" s="8"/>
-      <c r="J135" s="5"/>
-      <c r="K135" s="5"/>
-      <c r="L135" s="5"/>
-      <c r="M135" s="5"/>
-      <c r="N135" s="5"/>
+      <c r="B135" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="C135" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="D135" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="E135" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="F135" s="9">
+        <v>3.9</v>
+      </c>
+      <c r="G135" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="H135" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="I135" s="21" t="s">
+        <v>279</v>
+      </c>
+      <c r="J135" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="K135" s="5">
+        <v>0.3</v>
+      </c>
+      <c r="L135" s="5">
+        <v>0.3</v>
+      </c>
+      <c r="M135" s="5">
+        <v>0.6</v>
+      </c>
+      <c r="N135" s="5">
+        <v>0</v>
+      </c>
       <c r="O135" s="5"/>
       <c r="P135" s="5"/>
       <c r="Q135" s="5"/>
@@ -9567,11 +9791,43 @@
     </row>
     <row r="136" spans="1:24" ht="13.75" customHeight="1">
       <c r="A136" s="9"/>
-      <c r="J136" s="5"/>
-      <c r="K136" s="5"/>
-      <c r="L136" s="5"/>
-      <c r="M136" s="5"/>
-      <c r="N136" s="5"/>
+      <c r="B136" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="C136" s="8" t="s">
+        <v>256</v>
+      </c>
+      <c r="D136" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="E136" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="F136" s="9">
+        <v>2.5</v>
+      </c>
+      <c r="G136" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H136" s="12"/>
+      <c r="I136" s="21" t="s">
+        <v>275</v>
+      </c>
+      <c r="J136" s="5">
+        <v>0.4</v>
+      </c>
+      <c r="K136" s="5">
+        <v>0.4</v>
+      </c>
+      <c r="L136" s="5">
+        <v>0.3</v>
+      </c>
+      <c r="M136" s="5">
+        <v>0.8</v>
+      </c>
+      <c r="N136" s="5">
+        <v>0</v>
+      </c>
       <c r="O136" s="5"/>
       <c r="P136" s="5"/>
       <c r="Q136" s="5"/>
@@ -9584,12 +9840,44 @@
       <c r="X136" s="5"/>
     </row>
     <row r="137" spans="1:24" ht="13.75" customHeight="1">
-      <c r="A137" s="9"/>
-      <c r="J137" s="5"/>
-      <c r="K137" s="5"/>
-      <c r="L137" s="5"/>
-      <c r="M137" s="5"/>
-      <c r="N137" s="5"/>
+      <c r="A137"/>
+      <c r="B137" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="C137" s="8" t="s">
+        <v>260</v>
+      </c>
+      <c r="D137" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="E137" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="F137" s="9">
+        <v>2.9</v>
+      </c>
+      <c r="G137" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="H137" s="8"/>
+      <c r="I137" s="21" t="s">
+        <v>279</v>
+      </c>
+      <c r="J137" s="5">
+        <v>0.6</v>
+      </c>
+      <c r="K137" s="5">
+        <v>0.3</v>
+      </c>
+      <c r="L137" s="5">
+        <v>0.2</v>
+      </c>
+      <c r="M137" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="N137" s="5">
+        <v>0</v>
+      </c>
       <c r="O137" s="5"/>
       <c r="P137" s="5"/>
       <c r="Q137" s="5"/>
@@ -9603,11 +9891,45 @@
     </row>
     <row r="138" spans="1:24" ht="13.75" customHeight="1">
       <c r="A138" s="9"/>
-      <c r="J138" s="5"/>
-      <c r="K138" s="5"/>
-      <c r="L138" s="5"/>
-      <c r="M138" s="5"/>
-      <c r="N138" s="5"/>
+      <c r="B138" s="8" t="s">
+        <v>497</v>
+      </c>
+      <c r="C138" s="8" t="s">
+        <v>498</v>
+      </c>
+      <c r="D138" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="E138" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="F138" s="9">
+        <v>3.9</v>
+      </c>
+      <c r="G138" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="H138" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="I138" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="J138" s="5">
+        <v>0.6</v>
+      </c>
+      <c r="K138" s="5">
+        <v>0.6</v>
+      </c>
+      <c r="L138" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="M138" s="5">
+        <v>0.9</v>
+      </c>
+      <c r="N138" s="5">
+        <v>0</v>
+      </c>
       <c r="O138" s="5"/>
       <c r="P138" s="5"/>
       <c r="Q138" s="5"/>
@@ -9621,11 +9943,45 @@
     </row>
     <row r="139" spans="1:24" ht="13.75" customHeight="1">
       <c r="A139" s="9"/>
-      <c r="J139" s="5"/>
-      <c r="K139" s="5"/>
-      <c r="L139" s="5"/>
-      <c r="M139" s="5"/>
-      <c r="N139" s="5"/>
+      <c r="B139" s="8" t="s">
+        <v>499</v>
+      </c>
+      <c r="C139" s="8" t="s">
+        <v>500</v>
+      </c>
+      <c r="D139" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="E139" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="F139" s="9">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="G139" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H139" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="I139" s="8" t="s">
+        <v>281</v>
+      </c>
+      <c r="J139" s="5">
+        <v>0.7</v>
+      </c>
+      <c r="K139" s="5">
+        <v>0.6</v>
+      </c>
+      <c r="L139" s="5">
+        <v>0.6</v>
+      </c>
+      <c r="M139" s="5">
+        <v>0.8</v>
+      </c>
+      <c r="N139" s="5">
+        <v>0</v>
+      </c>
       <c r="O139" s="5"/>
       <c r="P139" s="5"/>
       <c r="Q139" s="5"/>
@@ -9639,11 +9995,43 @@
     </row>
     <row r="140" spans="1:24" ht="13.75" customHeight="1">
       <c r="A140" s="9"/>
-      <c r="J140" s="5"/>
-      <c r="K140" s="5"/>
-      <c r="L140" s="5"/>
-      <c r="M140" s="5"/>
-      <c r="N140" s="5"/>
+      <c r="B140" s="8" t="s">
+        <v>501</v>
+      </c>
+      <c r="C140" s="8" t="s">
+        <v>502</v>
+      </c>
+      <c r="D140" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="E140" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="F140" s="9">
+        <v>3.9</v>
+      </c>
+      <c r="G140" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="H140" s="8"/>
+      <c r="I140" s="8" t="s">
+        <v>281</v>
+      </c>
+      <c r="J140" s="5">
+        <v>0.6</v>
+      </c>
+      <c r="K140" s="5">
+        <v>0.3</v>
+      </c>
+      <c r="L140" s="5">
+        <v>0.3</v>
+      </c>
+      <c r="M140" s="5">
+        <v>0.8</v>
+      </c>
+      <c r="N140" s="5">
+        <v>0</v>
+      </c>
       <c r="O140" s="5"/>
       <c r="P140" s="5"/>
       <c r="Q140" s="5"/>
@@ -9657,11 +10045,43 @@
     </row>
     <row r="141" spans="1:24" ht="13.75" customHeight="1">
       <c r="A141" s="9"/>
-      <c r="J141" s="5"/>
-      <c r="K141" s="5"/>
-      <c r="L141" s="5"/>
-      <c r="M141" s="5"/>
-      <c r="N141" s="5"/>
+      <c r="B141" s="8" t="s">
+        <v>503</v>
+      </c>
+      <c r="C141" s="8" t="s">
+        <v>504</v>
+      </c>
+      <c r="D141" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="E141" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="F141" s="9">
+        <v>3.9</v>
+      </c>
+      <c r="G141" s="8" t="s">
+        <v>490</v>
+      </c>
+      <c r="H141" s="8"/>
+      <c r="I141" s="8" t="s">
+        <v>281</v>
+      </c>
+      <c r="J141" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="K141" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="L141" s="5">
+        <v>0.4</v>
+      </c>
+      <c r="M141" s="5">
+        <v>0.9</v>
+      </c>
+      <c r="N141" s="5">
+        <v>0</v>
+      </c>
       <c r="O141" s="5"/>
       <c r="P141" s="5"/>
       <c r="Q141" s="5"/>
@@ -9675,11 +10095,41 @@
     </row>
     <row r="142" spans="1:24" ht="13.75" customHeight="1">
       <c r="A142" s="9"/>
-      <c r="J142" s="5"/>
-      <c r="K142" s="5"/>
-      <c r="L142" s="5"/>
-      <c r="M142" s="5"/>
-      <c r="N142" s="5"/>
+      <c r="B142" s="8" t="s">
+        <v>505</v>
+      </c>
+      <c r="C142" s="8" t="s">
+        <v>506</v>
+      </c>
+      <c r="D142" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="E142" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="F142" s="9">
+        <v>3.9</v>
+      </c>
+      <c r="G142" s="8"/>
+      <c r="H142" s="8"/>
+      <c r="I142" s="8" t="s">
+        <v>278</v>
+      </c>
+      <c r="J142" s="5">
+        <v>0.6</v>
+      </c>
+      <c r="K142" s="5">
+        <v>0.4</v>
+      </c>
+      <c r="L142" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="M142" s="5">
+        <v>0.8</v>
+      </c>
+      <c r="N142" s="5">
+        <v>0</v>
+      </c>
       <c r="O142" s="5"/>
       <c r="P142" s="5"/>
       <c r="Q142" s="5"/>
@@ -9693,11 +10143,43 @@
     </row>
     <row r="143" spans="1:24" ht="13.75" customHeight="1">
       <c r="A143" s="9"/>
-      <c r="J143" s="5"/>
-      <c r="K143" s="5"/>
-      <c r="L143" s="5"/>
-      <c r="M143" s="5"/>
-      <c r="N143" s="5"/>
+      <c r="B143" s="8" t="s">
+        <v>507</v>
+      </c>
+      <c r="C143" s="8" t="s">
+        <v>508</v>
+      </c>
+      <c r="D143" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="E143" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="F143" s="9">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="G143" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="H143" s="8"/>
+      <c r="I143" s="8" t="s">
+        <v>278</v>
+      </c>
+      <c r="J143" s="5">
+        <v>0.8</v>
+      </c>
+      <c r="K143" s="5">
+        <v>0.3</v>
+      </c>
+      <c r="L143" s="5">
+        <v>0.3</v>
+      </c>
+      <c r="M143" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="N143" s="5">
+        <v>0</v>
+      </c>
       <c r="O143" s="5"/>
       <c r="P143" s="5"/>
       <c r="Q143" s="5"/>
@@ -9711,11 +10193,41 @@
     </row>
     <row r="144" spans="1:24" ht="13.75" customHeight="1">
       <c r="A144" s="9"/>
-      <c r="J144" s="5"/>
-      <c r="K144" s="5"/>
-      <c r="L144" s="5"/>
-      <c r="M144" s="5"/>
-      <c r="N144" s="5"/>
+      <c r="B144" s="8" t="s">
+        <v>509</v>
+      </c>
+      <c r="C144" s="8" t="s">
+        <v>510</v>
+      </c>
+      <c r="D144" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="E144" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="F144" s="9">
+        <v>3.9</v>
+      </c>
+      <c r="G144" s="8"/>
+      <c r="H144" s="8"/>
+      <c r="I144" s="8" t="s">
+        <v>278</v>
+      </c>
+      <c r="J144" s="5">
+        <v>0.7</v>
+      </c>
+      <c r="K144" s="5">
+        <v>0.3</v>
+      </c>
+      <c r="L144" s="5">
+        <v>0.3</v>
+      </c>
+      <c r="M144" s="5">
+        <v>0.7</v>
+      </c>
+      <c r="N144" s="5">
+        <v>0</v>
+      </c>
       <c r="O144" s="5"/>
       <c r="P144" s="5"/>
       <c r="Q144" s="5"/>
@@ -9729,6 +10241,13 @@
     </row>
     <row r="145" spans="1:24" ht="13.75" customHeight="1">
       <c r="A145" s="9"/>
+      <c r="B145" s="8"/>
+      <c r="C145" s="8"/>
+      <c r="D145" s="8"/>
+      <c r="E145" s="8"/>
+      <c r="F145" s="9"/>
+      <c r="G145" s="8"/>
+      <c r="H145" s="8"/>
       <c r="J145" s="5"/>
       <c r="K145" s="5"/>
       <c r="L145" s="5"/>
@@ -9747,6 +10266,13 @@
     </row>
     <row r="146" spans="1:24" ht="13.75" customHeight="1">
       <c r="A146" s="9"/>
+      <c r="B146" s="8"/>
+      <c r="C146" s="8"/>
+      <c r="D146" s="8"/>
+      <c r="E146" s="8"/>
+      <c r="F146" s="9"/>
+      <c r="G146" s="8"/>
+      <c r="H146" s="8"/>
       <c r="J146" s="5"/>
       <c r="K146" s="5"/>
       <c r="L146" s="5"/>
@@ -9765,6 +10291,14 @@
     </row>
     <row r="147" spans="1:24" ht="13.75" customHeight="1">
       <c r="A147" s="9"/>
+      <c r="B147" s="8"/>
+      <c r="C147" s="8"/>
+      <c r="D147" s="8"/>
+      <c r="E147" s="8"/>
+      <c r="F147" s="9"/>
+      <c r="G147" s="8"/>
+      <c r="H147" s="8"/>
+      <c r="I147" s="8"/>
       <c r="J147" s="5"/>
       <c r="K147" s="5"/>
       <c r="L147" s="5"/>
@@ -9783,6 +10317,14 @@
     </row>
     <row r="148" spans="1:24" ht="13.75" customHeight="1">
       <c r="A148" s="9"/>
+      <c r="B148" s="8"/>
+      <c r="C148" s="8"/>
+      <c r="D148" s="8"/>
+      <c r="E148" s="8"/>
+      <c r="F148" s="9"/>
+      <c r="G148" s="8"/>
+      <c r="H148" s="8"/>
+      <c r="I148" s="8"/>
       <c r="J148" s="5"/>
       <c r="K148" s="5"/>
       <c r="L148" s="5"/>
@@ -9801,6 +10343,14 @@
     </row>
     <row r="149" spans="1:24" ht="13.75" customHeight="1">
       <c r="A149" s="9"/>
+      <c r="B149" s="8"/>
+      <c r="C149" s="8"/>
+      <c r="D149" s="8"/>
+      <c r="E149" s="8"/>
+      <c r="F149" s="9"/>
+      <c r="G149" s="8"/>
+      <c r="H149" s="8"/>
+      <c r="I149" s="8"/>
       <c r="J149" s="5"/>
       <c r="K149" s="5"/>
       <c r="L149" s="5"/>
@@ -9819,6 +10369,14 @@
     </row>
     <row r="150" spans="1:24" ht="13.75" customHeight="1">
       <c r="A150" s="9"/>
+      <c r="B150" s="8"/>
+      <c r="C150" s="8"/>
+      <c r="D150" s="8"/>
+      <c r="E150" s="8"/>
+      <c r="F150" s="9"/>
+      <c r="G150" s="8"/>
+      <c r="H150" s="8"/>
+      <c r="I150" s="8"/>
       <c r="J150" s="5"/>
       <c r="K150" s="5"/>
       <c r="L150" s="5"/>
@@ -9837,6 +10395,14 @@
     </row>
     <row r="151" spans="1:24" ht="13.75" customHeight="1">
       <c r="A151" s="9"/>
+      <c r="B151" s="8"/>
+      <c r="C151" s="8"/>
+      <c r="D151" s="8"/>
+      <c r="E151" s="8"/>
+      <c r="F151" s="9"/>
+      <c r="G151" s="8"/>
+      <c r="H151" s="8"/>
+      <c r="I151" s="8"/>
       <c r="J151" s="5"/>
       <c r="K151" s="5"/>
       <c r="L151" s="5"/>
@@ -9855,6 +10421,14 @@
     </row>
     <row r="152" spans="1:24" ht="13.75" customHeight="1">
       <c r="A152" s="9"/>
+      <c r="B152" s="8"/>
+      <c r="C152" s="8"/>
+      <c r="D152" s="8"/>
+      <c r="E152" s="8"/>
+      <c r="F152" s="9"/>
+      <c r="G152" s="8"/>
+      <c r="H152" s="8"/>
+      <c r="I152" s="8"/>
       <c r="J152" s="5"/>
       <c r="K152" s="5"/>
       <c r="L152" s="5"/>
@@ -9873,6 +10447,13 @@
     </row>
     <row r="153" spans="1:24" ht="13.75" customHeight="1">
       <c r="A153" s="9"/>
+      <c r="B153" s="8"/>
+      <c r="C153" s="8"/>
+      <c r="D153" s="8"/>
+      <c r="E153" s="8"/>
+      <c r="F153" s="9"/>
+      <c r="G153" s="8"/>
+      <c r="H153" s="8"/>
       <c r="J153" s="5"/>
       <c r="K153" s="5"/>
       <c r="L153" s="5"/>
@@ -9891,6 +10472,14 @@
     </row>
     <row r="154" spans="1:24" ht="13.75" customHeight="1">
       <c r="A154" s="9"/>
+      <c r="B154" s="8"/>
+      <c r="C154" s="8"/>
+      <c r="D154" s="8"/>
+      <c r="E154" s="8"/>
+      <c r="F154" s="9"/>
+      <c r="G154" s="8"/>
+      <c r="H154" s="8"/>
+      <c r="I154" s="8"/>
       <c r="J154" s="5"/>
       <c r="K154" s="5"/>
       <c r="L154" s="5"/>
@@ -9909,6 +10498,14 @@
     </row>
     <row r="155" spans="1:24" ht="13.75" customHeight="1">
       <c r="A155" s="9"/>
+      <c r="B155" s="8"/>
+      <c r="C155" s="8"/>
+      <c r="D155" s="8"/>
+      <c r="E155" s="8"/>
+      <c r="F155" s="9"/>
+      <c r="G155" s="8"/>
+      <c r="H155" s="8"/>
+      <c r="I155" s="8"/>
       <c r="J155" s="5"/>
       <c r="K155" s="5"/>
       <c r="L155" s="5"/>
@@ -9927,6 +10524,14 @@
     </row>
     <row r="156" spans="1:24" ht="13.75" customHeight="1">
       <c r="A156" s="9"/>
+      <c r="B156" s="8"/>
+      <c r="C156" s="8"/>
+      <c r="D156" s="8"/>
+      <c r="E156" s="8"/>
+      <c r="F156" s="9"/>
+      <c r="G156" s="8"/>
+      <c r="H156" s="8"/>
+      <c r="I156" s="8"/>
       <c r="J156" s="5"/>
       <c r="K156" s="5"/>
       <c r="L156" s="5"/>
@@ -9945,6 +10550,14 @@
     </row>
     <row r="157" spans="1:24" ht="13.75" customHeight="1">
       <c r="A157" s="9"/>
+      <c r="B157" s="8"/>
+      <c r="C157" s="8"/>
+      <c r="D157" s="8"/>
+      <c r="E157" s="8"/>
+      <c r="F157" s="9"/>
+      <c r="G157" s="8"/>
+      <c r="H157" s="8"/>
+      <c r="I157" s="8"/>
       <c r="J157" s="5"/>
       <c r="K157" s="5"/>
       <c r="L157" s="5"/>
@@ -9963,6 +10576,14 @@
     </row>
     <row r="158" spans="1:24" ht="13.75" customHeight="1">
       <c r="A158" s="9"/>
+      <c r="B158" s="8"/>
+      <c r="C158" s="8"/>
+      <c r="D158" s="8"/>
+      <c r="E158" s="8"/>
+      <c r="F158" s="9"/>
+      <c r="G158" s="8"/>
+      <c r="H158" s="8"/>
+      <c r="I158" s="8"/>
       <c r="J158" s="5"/>
       <c r="K158" s="5"/>
       <c r="L158" s="5"/>
@@ -9981,6 +10602,14 @@
     </row>
     <row r="159" spans="1:24" ht="13.75" customHeight="1">
       <c r="A159" s="9"/>
+      <c r="B159" s="8"/>
+      <c r="C159" s="8"/>
+      <c r="D159" s="8"/>
+      <c r="E159" s="8"/>
+      <c r="F159" s="9"/>
+      <c r="G159" s="8"/>
+      <c r="H159" s="8"/>
+      <c r="I159" s="8"/>
       <c r="J159" s="5"/>
       <c r="K159" s="5"/>
       <c r="L159" s="5"/>
@@ -9999,6 +10628,13 @@
     </row>
     <row r="160" spans="1:24" ht="13.75" customHeight="1">
       <c r="A160" s="9"/>
+      <c r="B160" s="8"/>
+      <c r="C160" s="8"/>
+      <c r="D160" s="8"/>
+      <c r="E160" s="8"/>
+      <c r="F160" s="9"/>
+      <c r="G160" s="8"/>
+      <c r="H160" s="8"/>
       <c r="J160" s="5"/>
       <c r="K160" s="5"/>
       <c r="L160" s="5"/>
@@ -10017,6 +10653,14 @@
     </row>
     <row r="161" spans="1:24" ht="13.75" customHeight="1">
       <c r="A161" s="9"/>
+      <c r="B161" s="8"/>
+      <c r="C161" s="8"/>
+      <c r="D161" s="8"/>
+      <c r="E161" s="8"/>
+      <c r="F161" s="9"/>
+      <c r="G161" s="8"/>
+      <c r="H161" s="8"/>
+      <c r="I161" s="8"/>
       <c r="J161" s="5"/>
       <c r="K161" s="5"/>
       <c r="L161" s="5"/>
@@ -10035,6 +10679,14 @@
     </row>
     <row r="162" spans="1:24" ht="13.75" customHeight="1">
       <c r="A162" s="9"/>
+      <c r="B162" s="8"/>
+      <c r="C162" s="8"/>
+      <c r="D162" s="8"/>
+      <c r="E162" s="8"/>
+      <c r="F162" s="9"/>
+      <c r="G162" s="8"/>
+      <c r="H162" s="8"/>
+      <c r="I162" s="8"/>
       <c r="J162" s="5"/>
       <c r="K162" s="5"/>
       <c r="L162" s="5"/>
@@ -10053,6 +10705,14 @@
     </row>
     <row r="163" spans="1:24" ht="13.75" customHeight="1">
       <c r="A163" s="9"/>
+      <c r="B163" s="8"/>
+      <c r="C163" s="8"/>
+      <c r="D163" s="8"/>
+      <c r="E163" s="8"/>
+      <c r="F163" s="9"/>
+      <c r="G163" s="8"/>
+      <c r="H163" s="8"/>
+      <c r="I163" s="8"/>
       <c r="J163" s="5"/>
       <c r="K163" s="5"/>
       <c r="L163" s="5"/>
@@ -10071,6 +10731,14 @@
     </row>
     <row r="164" spans="1:24" ht="13.75" customHeight="1">
       <c r="A164" s="9"/>
+      <c r="B164" s="8"/>
+      <c r="C164" s="8"/>
+      <c r="D164" s="8"/>
+      <c r="E164" s="8"/>
+      <c r="F164" s="9"/>
+      <c r="G164" s="8"/>
+      <c r="H164" s="8"/>
+      <c r="I164" s="8"/>
       <c r="J164" s="5"/>
       <c r="K164" s="5"/>
       <c r="L164" s="5"/>
@@ -10089,6 +10757,14 @@
     </row>
     <row r="165" spans="1:24" ht="13.75" customHeight="1">
       <c r="A165" s="9"/>
+      <c r="B165" s="8"/>
+      <c r="C165" s="8"/>
+      <c r="D165" s="8"/>
+      <c r="E165" s="8"/>
+      <c r="F165" s="9"/>
+      <c r="G165" s="8"/>
+      <c r="H165" s="8"/>
+      <c r="I165" s="8"/>
       <c r="J165" s="5"/>
       <c r="K165" s="5"/>
       <c r="L165" s="5"/>
@@ -10107,6 +10783,14 @@
     </row>
     <row r="166" spans="1:24" ht="13.75" customHeight="1">
       <c r="A166" s="9"/>
+      <c r="B166" s="8"/>
+      <c r="C166" s="8"/>
+      <c r="D166" s="8"/>
+      <c r="E166" s="8"/>
+      <c r="F166" s="9"/>
+      <c r="G166" s="8"/>
+      <c r="H166" s="8"/>
+      <c r="I166" s="8"/>
       <c r="J166" s="5"/>
       <c r="K166" s="5"/>
       <c r="L166" s="5"/>
@@ -10125,6 +10809,13 @@
     </row>
     <row r="167" spans="1:24" ht="13.75" customHeight="1">
       <c r="A167" s="9"/>
+      <c r="B167" s="8"/>
+      <c r="C167" s="8"/>
+      <c r="D167" s="8"/>
+      <c r="E167" s="8"/>
+      <c r="F167" s="9"/>
+      <c r="G167" s="8"/>
+      <c r="H167" s="8"/>
       <c r="J167" s="5"/>
       <c r="K167" s="5"/>
       <c r="L167" s="5"/>
@@ -29977,8 +30668,14 @@
       <c r="X930" s="5"/>
     </row>
   </sheetData>
-  <autoFilter ref="B1:P128" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
-  <conditionalFormatting sqref="J2:N128">
+  <autoFilter ref="B1:P137" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="Dessert"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
+  <conditionalFormatting sqref="J2:N144">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -30002,6 +30699,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E21CFA1F-1FDA-B147-8AC7-55852FE3510B}">
   <dimension ref="B2:I33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13"/>
+  <cols>
+    <col min="2" max="2" width="27.83203125" customWidth="1"/>
+    <col min="3" max="3" width="39.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="2" spans="2:9" ht="16">
       <c r="B2" s="8" t="s">
@@ -30051,32 +30752,6 @@
       </c>
       <c r="I3" s="21"/>
     </row>
-    <row r="4" spans="2:9" ht="16">
-      <c r="B4" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>241</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>182</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" s="9">
-        <v>3.9</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="H4" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="I4" s="21" t="s">
-        <v>279</v>
-      </c>
-    </row>
     <row r="5" spans="2:9" ht="16">
       <c r="B5" s="8" t="s">
         <v>70</v>
@@ -30125,79 +30800,8 @@
       </c>
       <c r="I6" s="5"/>
     </row>
-    <row r="7" spans="2:9" ht="16">
-      <c r="B7" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>244</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>182</v>
-      </c>
-      <c r="E7" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" s="9">
-        <v>3.9</v>
-      </c>
-      <c r="G7" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="H7" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="I7" s="21"/>
-    </row>
-    <row r="8" spans="2:9" ht="16">
-      <c r="B8" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>245</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>182</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" s="9">
-        <v>3.9</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="H8" s="8" t="s">
-        <v>48</v>
-      </c>
+    <row r="8" spans="2:9">
       <c r="I8" s="5"/>
-    </row>
-    <row r="9" spans="2:9" ht="16">
-      <c r="B9" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>246</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>182</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F9" s="9">
-        <v>3.9</v>
-      </c>
-      <c r="G9" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="H9" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="I9" s="21" t="s">
-        <v>279</v>
-      </c>
     </row>
     <row r="10" spans="2:9" ht="16">
       <c r="B10" s="8" t="s">
@@ -30421,52 +31025,6 @@
       </c>
       <c r="I18" s="21"/>
     </row>
-    <row r="19" spans="2:9" ht="16">
-      <c r="B19" s="8" t="s">
-        <v>190</v>
-      </c>
-      <c r="C19" s="8" t="s">
-        <v>256</v>
-      </c>
-      <c r="D19" s="8" t="s">
-        <v>182</v>
-      </c>
-      <c r="E19" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F19" s="9">
-        <v>2.5</v>
-      </c>
-      <c r="G19" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="H19" s="12"/>
-      <c r="I19" s="5"/>
-    </row>
-    <row r="20" spans="2:9" ht="16">
-      <c r="B20" s="8" t="s">
-        <v>184</v>
-      </c>
-      <c r="C20" s="8" t="s">
-        <v>257</v>
-      </c>
-      <c r="D20" s="8" t="s">
-        <v>182</v>
-      </c>
-      <c r="E20" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F20" s="9">
-        <v>2.9</v>
-      </c>
-      <c r="G20" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="H20" s="12"/>
-      <c r="I20" s="21" t="s">
-        <v>275</v>
-      </c>
-    </row>
     <row r="21" spans="2:9" ht="16">
       <c r="B21" s="8" t="s">
         <v>183</v>
@@ -30513,28 +31071,6 @@
         <v>277</v>
       </c>
     </row>
-    <row r="23" spans="2:9" ht="16">
-      <c r="B23" s="8" t="s">
-        <v>191</v>
-      </c>
-      <c r="C23" s="8" t="s">
-        <v>260</v>
-      </c>
-      <c r="D23" s="8" t="s">
-        <v>182</v>
-      </c>
-      <c r="E23" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F23" s="9">
-        <v>2.9</v>
-      </c>
-      <c r="G23" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="H23" s="12"/>
-      <c r="I23" s="5"/>
-    </row>
     <row r="24" spans="2:9" ht="16">
       <c r="B24" s="8" t="s">
         <v>124</v>
@@ -30689,56 +31225,6 @@
       <c r="H30" s="12"/>
       <c r="I30" s="21" t="s">
         <v>276</v>
-      </c>
-    </row>
-    <row r="31" spans="2:9" ht="16">
-      <c r="B31" s="8" t="s">
-        <v>147</v>
-      </c>
-      <c r="C31" s="8" t="s">
-        <v>268</v>
-      </c>
-      <c r="D31" s="8" t="s">
-        <v>182</v>
-      </c>
-      <c r="E31" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F31" s="9">
-        <v>3.9</v>
-      </c>
-      <c r="G31" s="8" t="s">
-        <v>149</v>
-      </c>
-      <c r="H31" s="12"/>
-      <c r="I31" s="21" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="32" spans="2:9" ht="16">
-      <c r="B32" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="C32" s="8" t="s">
-        <v>269</v>
-      </c>
-      <c r="D32" s="8" t="s">
-        <v>182</v>
-      </c>
-      <c r="E32" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F32" s="9">
-        <v>3.9</v>
-      </c>
-      <c r="G32" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="H32" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="I32" s="21" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="33" spans="2:9" ht="16">

</xml_diff>